<commit_message>
SUM formula correcte; Headers Merged
</commit_message>
<xml_diff>
--- a/Deliverables/Interface_Board/BOM/Interface_Board_BOM Quantity(500).xlsx
+++ b/Deliverables/Interface_Board/BOM/Interface_Board_BOM Quantity(500).xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="270">
   <si>
     <t>Component list</t>
   </si>
@@ -803,9 +803,6 @@
     <t>IC</t>
   </si>
   <si>
-    <t xml:space="preserve">Is Part ki cost zayada ha kia hum is part ko local part se replays kr sakte han </t>
-  </si>
-  <si>
     <t>ARG05BTC9001N</t>
   </si>
   <si>
@@ -840,6 +837,12 @@
   </si>
   <si>
     <t>This header will be sourced in Control Board BOM</t>
+  </si>
+  <si>
+    <t>1 x 13p 510 pcs ordered from LCSC</t>
+  </si>
+  <si>
+    <t>2 x 13p 6 lots (100pcs / lot) ordered</t>
   </si>
 </sst>
 </file>
@@ -851,7 +854,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1034,14 +1037,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1388,7 +1383,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1596,12 +1591,6 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="18" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="20" fillId="4" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1711,19 +1700,7 @@
     <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1761,6 +1738,42 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="25" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1806,7 +1819,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2138,20 +2151,20 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="121"/>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
-      <c r="Q1" s="121"/>
-      <c r="R1" s="121"/>
-      <c r="S1" s="122"/>
+      <c r="K1" s="115"/>
+      <c r="L1" s="115"/>
+      <c r="M1" s="115"/>
+      <c r="N1" s="115"/>
+      <c r="O1" s="115"/>
+      <c r="P1" s="115"/>
+      <c r="Q1" s="115"/>
+      <c r="R1" s="115"/>
+      <c r="S1" s="116"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
-      <c r="C2" s="90"/>
+      <c r="C2" s="88"/>
       <c r="D2" s="10" t="s">
         <v>0</v>
       </c>
@@ -2176,7 +2189,7 @@
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
-      <c r="C3" s="91"/>
+      <c r="C3" s="89"/>
       <c r="D3" s="12" t="s">
         <v>1</v>
       </c>
@@ -2196,12 +2209,12 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="123"/>
+      <c r="S3" s="117"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
-      <c r="C4" s="91"/>
+      <c r="C4" s="89"/>
       <c r="D4" s="12" t="s">
         <v>2</v>
       </c>
@@ -2221,12 +2234,12 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="124"/>
+      <c r="S4" s="118"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
-      <c r="C5" s="91"/>
+      <c r="C5" s="89"/>
       <c r="D5" s="12" t="s">
         <v>3</v>
       </c>
@@ -2246,12 +2259,12 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="124"/>
+      <c r="S5" s="118"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
-      <c r="C6" s="92"/>
+      <c r="C6" s="90"/>
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
       <c r="F6" s="16"/>
@@ -2267,12 +2280,12 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="124"/>
+      <c r="S6" s="118"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
-      <c r="C7" s="93"/>
+      <c r="C7" s="91"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17"/>
       <c r="F7" s="18"/>
@@ -2288,12 +2301,12 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="124"/>
+      <c r="S7" s="118"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="25"/>
-      <c r="C8" s="94"/>
+      <c r="C8" s="92"/>
       <c r="D8" s="26"/>
       <c r="E8" s="26"/>
       <c r="F8" s="27"/>
@@ -2309,7 +2322,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="124"/>
+      <c r="S8" s="118"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2350,7 +2363,7 @@
         <v>191</v>
       </c>
       <c r="N9" s="28" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="O9" s="28" t="s">
         <v>192</v>
@@ -2374,7 +2387,7 @@
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="118" t="s">
+      <c r="C10" s="126" t="s">
         <v>248</v>
       </c>
       <c r="D10" s="41" t="s">
@@ -2414,7 +2427,7 @@
       <c r="O10" s="70" t="s">
         <v>197</v>
       </c>
-      <c r="P10" s="104">
+      <c r="P10" s="102">
         <v>2.3199999999999998E-2</v>
       </c>
       <c r="Q10" s="51">
@@ -2430,7 +2443,7 @@
         <f t="shared" ref="B11:B49" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="119"/>
+      <c r="C11" s="127"/>
       <c r="D11" s="45" t="s">
         <v>12</v>
       </c>
@@ -2440,7 +2453,7 @@
       <c r="F11" s="46" t="s">
         <v>93</v>
       </c>
-      <c r="G11" s="101" t="s">
+      <c r="G11" s="99" t="s">
         <v>120</v>
       </c>
       <c r="H11" s="45" t="s">
@@ -2468,7 +2481,7 @@
       <c r="O11" s="64" t="s">
         <v>197</v>
       </c>
-      <c r="P11" s="89">
+      <c r="P11" s="87">
         <v>1.4200000000000001E-2</v>
       </c>
       <c r="Q11" s="54">
@@ -2484,7 +2497,7 @@
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="119"/>
+      <c r="C12" s="127"/>
       <c r="D12" s="41" t="s">
         <v>13</v>
       </c>
@@ -2522,7 +2535,7 @@
       <c r="O12" s="71" t="s">
         <v>197</v>
       </c>
-      <c r="P12" s="104">
+      <c r="P12" s="102">
         <v>7.3599999999999999E-2</v>
       </c>
       <c r="Q12" s="51">
@@ -2538,7 +2551,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="119"/>
+      <c r="C13" s="127"/>
       <c r="D13" s="45" t="s">
         <v>14</v>
       </c>
@@ -2574,17 +2587,17 @@
         <v>1520</v>
       </c>
       <c r="O13" s="75" t="s">
-        <v>266</v>
-      </c>
-      <c r="P13" s="89">
+        <v>265</v>
+      </c>
+      <c r="P13" s="87">
         <v>0.1</v>
       </c>
       <c r="Q13" s="54">
         <f t="shared" si="2"/>
         <v>152</v>
       </c>
-      <c r="R13" s="114" t="s">
-        <v>267</v>
+      <c r="R13" s="112" t="s">
+        <v>266</v>
       </c>
       <c r="S13" s="49"/>
     </row>
@@ -2594,7 +2607,7 @@
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="119"/>
+      <c r="C14" s="127"/>
       <c r="D14" s="41" t="s">
         <v>15</v>
       </c>
@@ -2632,7 +2645,7 @@
       <c r="O14" s="73" t="s">
         <v>197</v>
       </c>
-      <c r="P14" s="104">
+      <c r="P14" s="102">
         <v>7.2999999999999995E-2</v>
       </c>
       <c r="Q14" s="51">
@@ -2648,7 +2661,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="119"/>
+      <c r="C15" s="127"/>
       <c r="D15" s="45" t="s">
         <v>16</v>
       </c>
@@ -2658,7 +2671,7 @@
       <c r="F15" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="G15" s="101" t="s">
+      <c r="G15" s="99" t="s">
         <v>122</v>
       </c>
       <c r="H15" s="45" t="s">
@@ -2686,7 +2699,7 @@
       <c r="O15" s="74" t="s">
         <v>197</v>
       </c>
-      <c r="P15" s="89">
+      <c r="P15" s="87">
         <v>2.5999999999999999E-3</v>
       </c>
       <c r="Q15" s="54">
@@ -2702,7 +2715,7 @@
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="119"/>
+      <c r="C16" s="127"/>
       <c r="D16" s="41" t="s">
         <v>17</v>
       </c>
@@ -2712,7 +2725,7 @@
       <c r="F16" s="42" t="s">
         <v>92</v>
       </c>
-      <c r="G16" s="102" t="s">
+      <c r="G16" s="100" t="s">
         <v>123</v>
       </c>
       <c r="H16" s="65" t="s">
@@ -2740,7 +2753,7 @@
       <c r="O16" s="71" t="s">
         <v>197</v>
       </c>
-      <c r="P16" s="104">
+      <c r="P16" s="102">
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="Q16" s="51">
@@ -2756,7 +2769,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="119"/>
+      <c r="C17" s="127"/>
       <c r="D17" s="45" t="s">
         <v>18</v>
       </c>
@@ -2794,7 +2807,7 @@
       <c r="O17" s="64" t="s">
         <v>197</v>
       </c>
-      <c r="P17" s="89">
+      <c r="P17" s="87">
         <v>9.4999999999999998E-3</v>
       </c>
       <c r="Q17" s="54">
@@ -2810,7 +2823,7 @@
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="119"/>
+      <c r="C18" s="127"/>
       <c r="D18" s="41" t="s">
         <v>19</v>
       </c>
@@ -2848,7 +2861,7 @@
       <c r="O18" s="73" t="s">
         <v>197</v>
       </c>
-      <c r="P18" s="104">
+      <c r="P18" s="102">
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="Q18" s="51">
@@ -2864,7 +2877,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="119"/>
+      <c r="C19" s="127"/>
       <c r="D19" s="45" t="s">
         <v>20</v>
       </c>
@@ -2902,7 +2915,7 @@
       <c r="O19" s="75" t="s">
         <v>197</v>
       </c>
-      <c r="P19" s="89">
+      <c r="P19" s="87">
         <v>1.6400000000000001E-2</v>
       </c>
       <c r="Q19" s="54">
@@ -2918,7 +2931,7 @@
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="120"/>
+      <c r="C20" s="128"/>
       <c r="D20" s="41" t="s">
         <v>21</v>
       </c>
@@ -2956,14 +2969,14 @@
       <c r="O20" s="73" t="s">
         <v>197</v>
       </c>
-      <c r="P20" s="104">
+      <c r="P20" s="102">
         <v>7.7200000000000005E-2</v>
       </c>
       <c r="Q20" s="51">
         <f t="shared" si="2"/>
         <v>78.744</v>
       </c>
-      <c r="R20" s="115" t="s">
+      <c r="R20" s="113" t="s">
         <v>204</v>
       </c>
       <c r="S20" s="57"/>
@@ -2974,7 +2987,7 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="119" t="s">
+      <c r="C21" s="127" t="s">
         <v>249</v>
       </c>
       <c r="D21" s="45" t="s">
@@ -3014,7 +3027,7 @@
       <c r="O21" s="75" t="s">
         <v>197</v>
       </c>
-      <c r="P21" s="89">
+      <c r="P21" s="87">
         <v>0.26669999999999999</v>
       </c>
       <c r="Q21" s="54">
@@ -3030,7 +3043,7 @@
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="119"/>
+      <c r="C22" s="127"/>
       <c r="D22" s="41" t="s">
         <v>23</v>
       </c>
@@ -3068,14 +3081,14 @@
       <c r="O22" s="67" t="s">
         <v>197</v>
       </c>
-      <c r="P22" s="104">
+      <c r="P22" s="102">
         <v>2.6100000000000002E-2</v>
       </c>
       <c r="Q22" s="51">
         <f t="shared" si="2"/>
         <v>13.572000000000001</v>
       </c>
-      <c r="R22" s="115"/>
+      <c r="R22" s="113"/>
       <c r="S22" s="57"/>
     </row>
     <row r="23" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3084,7 +3097,7 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="119"/>
+      <c r="C23" s="127"/>
       <c r="D23" s="45" t="s">
         <v>24</v>
       </c>
@@ -3122,7 +3135,7 @@
       <c r="O23" s="75" t="s">
         <v>197</v>
       </c>
-      <c r="P23" s="89">
+      <c r="P23" s="87">
         <v>1.78E-2</v>
       </c>
       <c r="Q23" s="54">
@@ -3138,7 +3151,7 @@
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="119"/>
+      <c r="C24" s="127"/>
       <c r="D24" s="41" t="s">
         <v>25</v>
       </c>
@@ -3176,7 +3189,7 @@
       <c r="O24" s="70" t="s">
         <v>197</v>
       </c>
-      <c r="P24" s="104">
+      <c r="P24" s="102">
         <v>5.6599999999999998E-2</v>
       </c>
       <c r="Q24" s="51">
@@ -3192,16 +3205,16 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="118" t="s">
+      <c r="C25" s="126" t="s">
         <v>250</v>
       </c>
       <c r="D25" s="45" t="s">
         <v>26</v>
       </c>
       <c r="E25" s="45" t="s">
-        <v>263</v>
-      </c>
-      <c r="F25" s="98" t="s">
+        <v>262</v>
+      </c>
+      <c r="F25" s="96" t="s">
         <v>201</v>
       </c>
       <c r="G25" s="45" t="s">
@@ -3227,20 +3240,22 @@
         <v>500</v>
       </c>
       <c r="N25" s="47">
-        <v>600</v>
+        <v>6</v>
       </c>
       <c r="O25" s="75" t="s">
         <v>239</v>
       </c>
-      <c r="P25" s="89">
-        <v>0.32579999999999998</v>
+      <c r="P25" s="87">
+        <v>35</v>
       </c>
       <c r="Q25" s="54">
-        <f t="shared" si="2"/>
-        <v>195.48</v>
+        <f>P25*N25</f>
+        <v>210</v>
       </c>
       <c r="R25" s="45"/>
-      <c r="S25" s="49"/>
+      <c r="S25" s="112" t="s">
+        <v>269</v>
+      </c>
     </row>
     <row r="26" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
@@ -3248,14 +3263,14 @@
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="119"/>
+      <c r="C26" s="127"/>
       <c r="D26" s="41" t="s">
         <v>27</v>
       </c>
       <c r="E26" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="F26" s="99" t="s">
+      <c r="F26" s="97" t="s">
         <v>201</v>
       </c>
       <c r="G26" s="41" t="s">
@@ -3286,7 +3301,7 @@
       <c r="O26" s="63" t="s">
         <v>197</v>
       </c>
-      <c r="P26" s="104">
+      <c r="P26" s="102">
         <v>1.2641</v>
       </c>
       <c r="Q26" s="51">
@@ -3302,14 +3317,14 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="120"/>
+      <c r="C27" s="128"/>
       <c r="D27" s="45" t="s">
         <v>28</v>
       </c>
       <c r="E27" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="F27" s="98" t="s">
+      <c r="F27" s="96" t="s">
         <v>201</v>
       </c>
       <c r="G27" s="45" t="s">
@@ -3338,11 +3353,11 @@
         <v>510</v>
       </c>
       <c r="O27" s="55"/>
-      <c r="P27" s="89"/>
+      <c r="P27" s="87"/>
       <c r="Q27" s="54"/>
       <c r="R27" s="45"/>
-      <c r="S27" s="114" t="s">
-        <v>268</v>
+      <c r="S27" s="112" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3351,7 +3366,7 @@
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="118" t="s">
+      <c r="C28" s="126" t="s">
         <v>251</v>
       </c>
       <c r="D28" s="41" t="s">
@@ -3360,7 +3375,7 @@
       <c r="E28" s="41" t="s">
         <v>69</v>
       </c>
-      <c r="F28" s="99" t="s">
+      <c r="F28" s="97" t="s">
         <v>201</v>
       </c>
       <c r="G28" s="41" t="s">
@@ -3391,7 +3406,7 @@
       <c r="O28" s="76" t="s">
         <v>197</v>
       </c>
-      <c r="P28" s="104">
+      <c r="P28" s="102">
         <v>3.8600000000000002E-2</v>
       </c>
       <c r="Q28" s="51">
@@ -3407,7 +3422,7 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="120"/>
+      <c r="C29" s="128"/>
       <c r="D29" s="45" t="s">
         <v>30</v>
       </c>
@@ -3443,17 +3458,17 @@
         <v>505</v>
       </c>
       <c r="O29" s="75" t="s">
-        <v>266</v>
-      </c>
-      <c r="P29" s="89">
+        <v>265</v>
+      </c>
+      <c r="P29" s="87">
         <v>0.73</v>
       </c>
       <c r="Q29" s="54">
         <f t="shared" si="2"/>
         <v>368.65</v>
       </c>
-      <c r="R29" s="114" t="s">
-        <v>267</v>
+      <c r="R29" s="112" t="s">
+        <v>266</v>
       </c>
       <c r="S29" s="49"/>
     </row>
@@ -3463,7 +3478,7 @@
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
-      <c r="C30" s="118" t="s">
+      <c r="C30" s="126" t="s">
         <v>250</v>
       </c>
       <c r="D30" s="41" t="s">
@@ -3497,29 +3512,31 @@
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="N30" s="41">
-        <v>520</v>
-      </c>
-      <c r="O30" s="77" t="s">
+      <c r="N30" s="130">
+        <v>500</v>
+      </c>
+      <c r="O30" s="131" t="s">
         <v>197</v>
       </c>
-      <c r="P30" s="104">
-        <v>2.47E-2</v>
-      </c>
-      <c r="Q30" s="51">
-        <f t="shared" si="2"/>
-        <v>12.843999999999999</v>
-      </c>
-      <c r="R30" s="41"/>
-      <c r="S30" s="57"/>
-    </row>
-    <row r="31" spans="1:19" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P30" s="133">
+        <v>8.8400000000000006E-2</v>
+      </c>
+      <c r="Q30" s="135">
+        <f>P30*N30</f>
+        <v>44.2</v>
+      </c>
+      <c r="R30" s="130"/>
+      <c r="S30" s="136" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="36">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="119"/>
+      <c r="C31" s="127"/>
       <c r="D31" s="45" t="s">
         <v>32</v>
       </c>
@@ -3551,23 +3568,12 @@
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="N31" s="47">
-        <v>1005</v>
-      </c>
-      <c r="O31" s="78" t="s">
-        <v>197</v>
-      </c>
-      <c r="P31" s="89">
-        <v>0.20269999999999999</v>
-      </c>
-      <c r="Q31" s="54">
-        <f t="shared" si="2"/>
-        <v>203.71349999999998</v>
-      </c>
-      <c r="R31" s="116" t="s">
-        <v>256</v>
-      </c>
-      <c r="S31" s="49"/>
+      <c r="N31" s="129"/>
+      <c r="O31" s="132"/>
+      <c r="P31" s="134"/>
+      <c r="Q31" s="134"/>
+      <c r="R31" s="129"/>
+      <c r="S31" s="137"/>
     </row>
     <row r="32" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
@@ -3575,8 +3581,8 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="97" t="s">
-        <v>265</v>
+      <c r="C32" s="95" t="s">
+        <v>264</v>
       </c>
       <c r="D32" s="41" t="s">
         <v>33</v>
@@ -3621,7 +3627,7 @@
       <c r="Q32" s="56" t="s">
         <v>202</v>
       </c>
-      <c r="R32" s="117" t="s">
+      <c r="R32" s="114" t="s">
         <v>231</v>
       </c>
       <c r="S32" s="57"/>
@@ -3632,7 +3638,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="96" t="s">
+      <c r="C33" s="94" t="s">
         <v>252</v>
       </c>
       <c r="D33" s="45" t="s">
@@ -3644,7 +3650,7 @@
       <c r="F33" s="46" t="s">
         <v>201</v>
       </c>
-      <c r="G33" s="103" t="s">
+      <c r="G33" s="101" t="s">
         <v>108</v>
       </c>
       <c r="H33" s="53" t="s">
@@ -3669,10 +3675,10 @@
       <c r="N33" s="45">
         <v>510</v>
       </c>
-      <c r="O33" s="79" t="s">
+      <c r="O33" s="77" t="s">
         <v>197</v>
       </c>
-      <c r="P33" s="89">
+      <c r="P33" s="87">
         <v>0.56630000000000003</v>
       </c>
       <c r="Q33" s="54">
@@ -3688,7 +3694,7 @@
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="97" t="s">
+      <c r="C34" s="95" t="s">
         <v>253</v>
       </c>
       <c r="D34" s="41" t="s">
@@ -3728,7 +3734,7 @@
       <c r="O34" s="70" t="s">
         <v>197</v>
       </c>
-      <c r="P34" s="104">
+      <c r="P34" s="102">
         <v>4.4699999999999997E-2</v>
       </c>
       <c r="Q34" s="51">
@@ -3744,7 +3750,7 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="118" t="s">
+      <c r="C35" s="126" t="s">
         <v>254</v>
       </c>
       <c r="D35" s="45" t="s">
@@ -3781,10 +3787,10 @@
       <c r="N35" s="47">
         <v>1600</v>
       </c>
-      <c r="O35" s="80" t="s">
+      <c r="O35" s="78" t="s">
         <v>197</v>
       </c>
-      <c r="P35" s="89">
+      <c r="P35" s="87">
         <v>1.6999999999999999E-3</v>
       </c>
       <c r="Q35" s="54">
@@ -3800,7 +3806,7 @@
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="119"/>
+      <c r="C36" s="127"/>
       <c r="D36" s="41" t="s">
         <v>37</v>
       </c>
@@ -3810,17 +3816,17 @@
       <c r="F36" s="42" t="s">
         <v>110</v>
       </c>
-      <c r="G36" s="102" t="s">
+      <c r="G36" s="100" t="s">
         <v>130</v>
       </c>
       <c r="H36" s="41" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I36" s="43" t="s">
         <v>153</v>
       </c>
       <c r="J36" s="41" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="K36" s="41" t="s">
         <v>178</v>
@@ -3838,7 +3844,7 @@
       <c r="O36" s="63" t="s">
         <v>197</v>
       </c>
-      <c r="P36" s="104">
+      <c r="P36" s="102">
         <v>1.4E-3</v>
       </c>
       <c r="Q36" s="51">
@@ -3854,7 +3860,7 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="119"/>
+      <c r="C37" s="127"/>
       <c r="D37" s="45" t="s">
         <v>38</v>
       </c>
@@ -3864,7 +3870,7 @@
       <c r="F37" s="46" t="s">
         <v>111</v>
       </c>
-      <c r="G37" s="101" t="s">
+      <c r="G37" s="99" t="s">
         <v>131</v>
       </c>
       <c r="H37" s="59" t="s">
@@ -3892,7 +3898,7 @@
       <c r="O37" s="72" t="s">
         <v>197</v>
       </c>
-      <c r="P37" s="89">
+      <c r="P37" s="87">
         <v>9.8699999999999996E-2</v>
       </c>
       <c r="Q37" s="54">
@@ -3908,7 +3914,7 @@
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
-      <c r="C38" s="119"/>
+      <c r="C38" s="127"/>
       <c r="D38" s="41" t="s">
         <v>39</v>
       </c>
@@ -3918,17 +3924,17 @@
       <c r="F38" s="42" t="s">
         <v>112</v>
       </c>
-      <c r="G38" s="102" t="s">
-        <v>260</v>
+      <c r="G38" s="100" t="s">
+        <v>259</v>
       </c>
       <c r="H38" s="41" t="s">
+        <v>256</v>
+      </c>
+      <c r="I38" s="43" t="s">
         <v>257</v>
       </c>
-      <c r="I38" s="43" t="s">
+      <c r="J38" s="41" t="s">
         <v>258</v>
-      </c>
-      <c r="J38" s="41" t="s">
-        <v>259</v>
       </c>
       <c r="K38" s="41" t="s">
         <v>180</v>
@@ -3946,7 +3952,7 @@
       <c r="O38" s="63" t="s">
         <v>197</v>
       </c>
-      <c r="P38" s="104">
+      <c r="P38" s="102">
         <v>3.2399999999999998E-2</v>
       </c>
       <c r="Q38" s="51">
@@ -3962,7 +3968,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="119"/>
+      <c r="C39" s="127"/>
       <c r="D39" s="45" t="s">
         <v>40</v>
       </c>
@@ -4000,7 +4006,7 @@
       <c r="O39" s="72" t="s">
         <v>197</v>
       </c>
-      <c r="P39" s="89">
+      <c r="P39" s="87">
         <v>1.2999999999999999E-3</v>
       </c>
       <c r="Q39" s="54">
@@ -4016,7 +4022,7 @@
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
-      <c r="C40" s="119"/>
+      <c r="C40" s="127"/>
       <c r="D40" s="41" t="s">
         <v>41</v>
       </c>
@@ -4051,10 +4057,10 @@
       <c r="N40" s="41">
         <v>4100</v>
       </c>
-      <c r="O40" s="81" t="s">
+      <c r="O40" s="79" t="s">
         <v>197</v>
       </c>
-      <c r="P40" s="104">
+      <c r="P40" s="102">
         <v>8.9999999999999998E-4</v>
       </c>
       <c r="Q40" s="51">
@@ -4070,7 +4076,7 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C41" s="119"/>
+      <c r="C41" s="127"/>
       <c r="D41" s="45" t="s">
         <v>42</v>
       </c>
@@ -4108,7 +4114,7 @@
       <c r="O41" s="72" t="s">
         <v>197</v>
       </c>
-      <c r="P41" s="89">
+      <c r="P41" s="87">
         <v>1E-3</v>
       </c>
       <c r="Q41" s="54">
@@ -4124,7 +4130,7 @@
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
-      <c r="C42" s="119"/>
+      <c r="C42" s="127"/>
       <c r="D42" s="41" t="s">
         <v>43</v>
       </c>
@@ -4159,10 +4165,10 @@
       <c r="N42" s="41">
         <v>520</v>
       </c>
-      <c r="O42" s="82" t="s">
+      <c r="O42" s="80" t="s">
         <v>197</v>
       </c>
-      <c r="P42" s="104">
+      <c r="P42" s="102">
         <v>2.46E-2</v>
       </c>
       <c r="Q42" s="51">
@@ -4178,7 +4184,7 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="119"/>
+      <c r="C43" s="127"/>
       <c r="D43" s="45" t="s">
         <v>44</v>
       </c>
@@ -4213,10 +4219,10 @@
       <c r="N43" s="47">
         <v>600</v>
       </c>
-      <c r="O43" s="83" t="s">
+      <c r="O43" s="81" t="s">
         <v>197</v>
       </c>
-      <c r="P43" s="89">
+      <c r="P43" s="87">
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="Q43" s="54">
@@ -4232,7 +4238,7 @@
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
-      <c r="C44" s="119"/>
+      <c r="C44" s="127"/>
       <c r="D44" s="41" t="s">
         <v>45</v>
       </c>
@@ -4270,7 +4276,7 @@
       <c r="O44" s="70" t="s">
         <v>197</v>
       </c>
-      <c r="P44" s="104">
+      <c r="P44" s="102">
         <v>1.2999999999999999E-3</v>
       </c>
       <c r="Q44" s="51">
@@ -4286,7 +4292,7 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C45" s="120"/>
+      <c r="C45" s="128"/>
       <c r="D45" s="45" t="s">
         <v>46</v>
       </c>
@@ -4321,10 +4327,10 @@
       <c r="N45" s="47">
         <v>1050</v>
       </c>
-      <c r="O45" s="83" t="s">
+      <c r="O45" s="81" t="s">
         <v>197</v>
       </c>
-      <c r="P45" s="89">
+      <c r="P45" s="87">
         <v>1.12E-2</v>
       </c>
       <c r="Q45" s="54">
@@ -4340,7 +4346,7 @@
         <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
-      <c r="C46" s="97" t="s">
+      <c r="C46" s="95" t="s">
         <v>114</v>
       </c>
       <c r="D46" s="41" t="s">
@@ -4380,13 +4386,13 @@
       <c r="O46" s="60" t="s">
         <v>202</v>
       </c>
-      <c r="P46" s="105" t="s">
+      <c r="P46" s="103" t="s">
         <v>202</v>
       </c>
       <c r="Q46" s="60" t="s">
         <v>202</v>
       </c>
-      <c r="R46" s="117" t="s">
+      <c r="R46" s="114" t="s">
         <v>231</v>
       </c>
       <c r="S46" s="60" t="s">
@@ -4399,7 +4405,7 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="119" t="s">
+      <c r="C47" s="127" t="s">
         <v>255</v>
       </c>
       <c r="D47" s="45" t="s">
@@ -4437,17 +4443,17 @@
         <v>505</v>
       </c>
       <c r="O47" s="75" t="s">
-        <v>266</v>
-      </c>
-      <c r="P47" s="89">
+        <v>265</v>
+      </c>
+      <c r="P47" s="87">
         <v>2.96</v>
       </c>
       <c r="Q47" s="52">
         <f t="shared" si="2"/>
         <v>1494.8</v>
       </c>
-      <c r="R47" s="114" t="s">
-        <v>267</v>
+      <c r="R47" s="112" t="s">
+        <v>266</v>
       </c>
       <c r="S47" s="49"/>
     </row>
@@ -4457,14 +4463,14 @@
         <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
-      <c r="C48" s="119"/>
+      <c r="C48" s="127"/>
       <c r="D48" s="41" t="s">
         <v>49</v>
       </c>
       <c r="E48" s="41" t="s">
         <v>89</v>
       </c>
-      <c r="F48" s="100" t="s">
+      <c r="F48" s="98" t="s">
         <v>232</v>
       </c>
       <c r="G48" s="41" t="s">
@@ -4492,10 +4498,10 @@
       <c r="N48" s="41">
         <v>505</v>
       </c>
-      <c r="O48" s="84" t="s">
+      <c r="O48" s="82" t="s">
         <v>197</v>
       </c>
-      <c r="P48" s="104">
+      <c r="P48" s="102">
         <v>3.1503999999999999</v>
       </c>
       <c r="Q48" s="51">
@@ -4511,7 +4517,7 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C49" s="120"/>
+      <c r="C49" s="128"/>
       <c r="D49" s="45" t="s">
         <v>50</v>
       </c>
@@ -4543,28 +4549,28 @@
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="N49" s="88">
+      <c r="N49" s="86">
         <v>505</v>
       </c>
       <c r="O49" s="75" t="s">
-        <v>266</v>
-      </c>
-      <c r="P49" s="89">
+        <v>265</v>
+      </c>
+      <c r="P49" s="87">
         <v>0.1</v>
       </c>
-      <c r="Q49" s="106">
+      <c r="Q49" s="104">
         <f t="shared" si="2"/>
         <v>50.5</v>
       </c>
-      <c r="R49" s="114" t="s">
-        <v>267</v>
+      <c r="R49" s="112" t="s">
+        <v>266</v>
       </c>
       <c r="S49" s="49"/>
     </row>
     <row r="50" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="31"/>
-      <c r="C50" s="95"/>
+      <c r="C50" s="93"/>
       <c r="D50" s="32" t="s">
         <v>5</v>
       </c>
@@ -4576,45 +4582,45 @@
       <c r="J50" s="34"/>
       <c r="K50" s="35"/>
       <c r="L50" s="35"/>
-      <c r="M50" s="107"/>
-      <c r="N50" s="125" t="s">
+      <c r="M50" s="105"/>
+      <c r="N50" s="119" t="s">
         <v>243</v>
       </c>
-      <c r="O50" s="126"/>
-      <c r="P50" s="126"/>
-      <c r="Q50" s="85">
+      <c r="O50" s="120"/>
+      <c r="P50" s="120"/>
+      <c r="Q50" s="83">
         <f>SUM(Q10:Q49)</f>
-        <v>6190.0655000000006</v>
-      </c>
-      <c r="R50" s="128"/>
-      <c r="S50" s="129"/>
+        <v>6032.228000000001</v>
+      </c>
+      <c r="R50" s="122"/>
+      <c r="S50" s="123"/>
     </row>
     <row r="51" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
-      <c r="B51" s="108"/>
-      <c r="C51" s="109"/>
+      <c r="B51" s="106"/>
+      <c r="C51" s="107"/>
       <c r="D51" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E51" s="110"/>
-      <c r="F51" s="111"/>
-      <c r="G51" s="112"/>
-      <c r="H51" s="112"/>
-      <c r="I51" s="111"/>
-      <c r="J51" s="111"/>
-      <c r="K51" s="112"/>
-      <c r="L51" s="112"/>
-      <c r="M51" s="113"/>
-      <c r="N51" s="125" t="s">
+      <c r="E51" s="108"/>
+      <c r="F51" s="109"/>
+      <c r="G51" s="110"/>
+      <c r="H51" s="110"/>
+      <c r="I51" s="109"/>
+      <c r="J51" s="109"/>
+      <c r="K51" s="110"/>
+      <c r="L51" s="110"/>
+      <c r="M51" s="111"/>
+      <c r="N51" s="119" t="s">
         <v>245</v>
       </c>
-      <c r="O51" s="126"/>
-      <c r="P51" s="127"/>
-      <c r="Q51" s="87">
-        <v>67.599999999999994</v>
-      </c>
-      <c r="R51" s="130"/>
-      <c r="S51" s="131"/>
+      <c r="O51" s="120"/>
+      <c r="P51" s="121"/>
+      <c r="Q51" s="85">
+        <v>80.599999999999994</v>
+      </c>
+      <c r="R51" s="124"/>
+      <c r="S51" s="125"/>
     </row>
     <row r="52" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
@@ -4628,24 +4634,18 @@
       <c r="K52" s="24"/>
       <c r="L52" s="24"/>
       <c r="M52" s="24"/>
-      <c r="N52" s="125" t="s">
+      <c r="N52" s="119" t="s">
         <v>244</v>
       </c>
-      <c r="O52" s="126"/>
-      <c r="P52" s="126"/>
-      <c r="Q52" s="86">
-        <f>Q50/500</f>
-        <v>12.380131</v>
+      <c r="O52" s="120"/>
+      <c r="P52" s="120"/>
+      <c r="Q52" s="84">
+        <f>SUM(Q50:Q51)/500</f>
+        <v>12.225656000000003</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="K1:S1"/>
-    <mergeCell ref="S3:S8"/>
-    <mergeCell ref="N50:P50"/>
-    <mergeCell ref="N52:P52"/>
-    <mergeCell ref="N51:P51"/>
-    <mergeCell ref="R50:S51"/>
+  <mergeCells count="19">
     <mergeCell ref="C35:C45"/>
     <mergeCell ref="C47:C49"/>
     <mergeCell ref="C10:C20"/>
@@ -4653,6 +4653,18 @@
     <mergeCell ref="C25:C27"/>
     <mergeCell ref="C28:C29"/>
     <mergeCell ref="C30:C31"/>
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N50:P50"/>
+    <mergeCell ref="N52:P52"/>
+    <mergeCell ref="N51:P51"/>
+    <mergeCell ref="R50:S51"/>
+    <mergeCell ref="N30:N31"/>
+    <mergeCell ref="O30:O31"/>
+    <mergeCell ref="P30:P31"/>
+    <mergeCell ref="Q30:Q31"/>
+    <mergeCell ref="S30:S31"/>
+    <mergeCell ref="R30:R31"/>
   </mergeCells>
   <conditionalFormatting sqref="O14">
     <cfRule type="dataBar" priority="15">
@@ -4865,10 +4877,10 @@
     <hyperlink ref="O22" r:id="rId26"/>
     <hyperlink ref="O26" r:id="rId27"/>
     <hyperlink ref="O30" r:id="rId28"/>
-    <hyperlink ref="O31" r:id="rId29"/>
-    <hyperlink ref="O25" r:id="rId30"/>
-    <hyperlink ref="O38" r:id="rId31"/>
-    <hyperlink ref="O36" r:id="rId32"/>
+    <hyperlink ref="O25" r:id="rId29"/>
+    <hyperlink ref="O38" r:id="rId30"/>
+    <hyperlink ref="O36" r:id="rId31"/>
+    <hyperlink ref="O30:O31" r:id="rId32" display="LCSC"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId33"/>

</xml_diff>